<commit_message>
Actualizo reportes y scripts de limpieza de datos
</commit_message>
<xml_diff>
--- a/ml/reports/conteo_cultivos_EVA.xlsx
+++ b/ml/reports/conteo_cultivos_EVA.xlsx
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>39390</v>
+        <v>39380</v>
       </c>
       <c r="C2" t="n">
         <v>1081</v>
@@ -495,10 +495,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15918</v>
+        <v>15871</v>
       </c>
       <c r="C3" t="n">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="D3" t="n">
         <v>18</v>
@@ -507,10 +507,10 @@
         <v>33</v>
       </c>
       <c r="F3" t="n">
-        <v>4010</v>
+        <v>4008</v>
       </c>
       <c r="G3" t="n">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="H3" t="n">
         <v>46</v>
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2435</v>
+        <v>2439</v>
       </c>
       <c r="C4" t="n">
         <v>158</v>
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>39390</v>
+        <v>39380</v>
       </c>
       <c r="C2" t="n">
         <v>1081</v>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>22015</v>
+        <v>22007</v>
       </c>
       <c r="C3" t="n">
         <v>860</v>
@@ -663,10 +663,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15918</v>
+        <v>15871</v>
       </c>
       <c r="C4" t="n">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="D4" t="n">
         <v>18</v>
@@ -675,10 +675,10 @@
         <v>33</v>
       </c>
       <c r="F4" t="n">
-        <v>4010</v>
+        <v>4008</v>
       </c>
       <c r="G4" t="n">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="H4" t="n">
         <v>46</v>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15590</v>
+        <v>15585</v>
       </c>
       <c r="C5" t="n">
         <v>668</v>
@@ -703,7 +703,7 @@
         <v>30</v>
       </c>
       <c r="F5" t="n">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="G5" t="n">
         <v>15</v>
@@ -719,7 +719,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13795</v>
+        <v>13796</v>
       </c>
       <c r="C6" t="n">
         <v>881</v>
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11566</v>
+        <v>11630</v>
       </c>
       <c r="C7" t="n">
         <v>344</v>
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10950</v>
+        <v>10953</v>
       </c>
       <c r="C8" t="n">
         <v>660</v>
@@ -859,10 +859,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9081</v>
+        <v>9077</v>
       </c>
       <c r="C11" t="n">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D11" t="n">
         <v>18</v>
@@ -871,7 +871,7 @@
         <v>31</v>
       </c>
       <c r="F11" t="n">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="G11" t="n">
         <v>308</v>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5133</v>
+        <v>5140</v>
       </c>
       <c r="C15" t="n">
         <v>587</v>
@@ -983,7 +983,7 @@
         <v>32</v>
       </c>
       <c r="F15" t="n">
-        <v>950</v>
+        <v>953</v>
       </c>
       <c r="G15" t="n">
         <v>121</v>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4191</v>
+        <v>4188</v>
       </c>
       <c r="C20" t="n">
         <v>405</v>
@@ -1139,7 +1139,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3950</v>
+        <v>3990</v>
       </c>
       <c r="C21" t="n">
         <v>637</v>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3777</v>
+        <v>3776</v>
       </c>
       <c r="C22" t="n">
         <v>265</v>
@@ -1179,7 +1179,7 @@
         <v>29</v>
       </c>
       <c r="F22" t="n">
-        <v>2297</v>
+        <v>2296</v>
       </c>
       <c r="G22" t="n">
         <v>207</v>
@@ -1251,16 +1251,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3664</v>
+        <v>3635</v>
       </c>
       <c r="C25" t="n">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D25" t="n">
         <v>18</v>
       </c>
       <c r="E25" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F25" t="n">
         <v>139</v>
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3451</v>
+        <v>3405</v>
       </c>
       <c r="C27" t="n">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D27" t="n">
         <v>18</v>
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3356</v>
+        <v>3373</v>
       </c>
       <c r="C28" t="n">
         <v>222</v>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3278</v>
+        <v>3274</v>
       </c>
       <c r="C29" t="n">
         <v>358</v>
@@ -1583,57 +1583,57 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AJI</t>
+          <t>GRANADILLA</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2607</v>
+        <v>2584</v>
       </c>
       <c r="C37" t="n">
-        <v>245</v>
+        <v>279</v>
       </c>
       <c r="D37" t="n">
         <v>18</v>
       </c>
       <c r="E37" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F37" t="n">
-        <v>1743</v>
+        <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>196</v>
+        <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GRANADILLA</t>
+          <t>AJI</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2550</v>
+        <v>2583</v>
       </c>
       <c r="C38" t="n">
-        <v>277</v>
+        <v>243</v>
       </c>
       <c r="D38" t="n">
         <v>18</v>
       </c>
       <c r="E38" t="n">
+        <v>27</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1743</v>
+      </c>
+      <c r="G38" t="n">
+        <v>196</v>
+      </c>
+      <c r="H38" t="n">
         <v>16</v>
-      </c>
-      <c r="F38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2500</v>
+        <v>2502</v>
       </c>
       <c r="C39" t="n">
         <v>357</v>
@@ -1671,10 +1671,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2450</v>
+        <v>2443</v>
       </c>
       <c r="C40" t="n">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D40" t="n">
         <v>18</v>
@@ -1683,7 +1683,7 @@
         <v>28</v>
       </c>
       <c r="F40" t="n">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G40" t="n">
         <v>26</v>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2435</v>
+        <v>2439</v>
       </c>
       <c r="C41" t="n">
         <v>158</v>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2260</v>
+        <v>2250</v>
       </c>
       <c r="C42" t="n">
         <v>239</v>
@@ -1739,7 +1739,7 @@
         <v>28</v>
       </c>
       <c r="F42" t="n">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G42" t="n">
         <v>52</v>
@@ -1755,10 +1755,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1943</v>
+        <v>1910</v>
       </c>
       <c r="C43" t="n">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D43" t="n">
         <v>18</v>
@@ -1767,10 +1767,10 @@
         <v>21</v>
       </c>
       <c r="F43" t="n">
-        <v>1017</v>
+        <v>994</v>
       </c>
       <c r="G43" t="n">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H43" t="n">
         <v>16</v>
@@ -1835,57 +1835,57 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>REPOLLO</t>
+          <t>OTRAS HORTALIZAS</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1677</v>
+        <v>1671</v>
       </c>
       <c r="C46" t="n">
-        <v>126</v>
+        <v>193</v>
       </c>
       <c r="D46" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E46" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F46" t="n">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OTRAS HORTALIZAS</t>
+          <t>REPOLLO</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1671</v>
+        <v>1651</v>
       </c>
       <c r="C47" t="n">
-        <v>193</v>
+        <v>123</v>
       </c>
       <c r="D47" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E47" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F47" t="n">
-        <v>69</v>
+        <v>2</v>
       </c>
       <c r="G47" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="C52" t="n">
         <v>111</v>
@@ -2091,7 +2091,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="C55" t="n">
         <v>167</v>
@@ -2103,7 +2103,7 @@
         <v>15</v>
       </c>
       <c r="F55" t="n">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="G55" t="n">
         <v>52</v>
@@ -2119,10 +2119,10 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1035</v>
+        <v>1050</v>
       </c>
       <c r="C56" t="n">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D56" t="n">
         <v>18</v>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>850</v>
+        <v>817</v>
       </c>
       <c r="C62" t="n">
         <v>69</v>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="C68" t="n">
         <v>74</v>
@@ -2467,7 +2467,7 @@
         <v>11</v>
       </c>
       <c r="F68" t="n">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G68" t="n">
         <v>93</v>
@@ -2623,10 +2623,10 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C74" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D74" t="n">
         <v>6</v>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>586</v>
+        <v>575</v>
       </c>
       <c r="C76" t="n">
         <v>58</v>
@@ -2707,10 +2707,10 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>569</v>
+        <v>557</v>
       </c>
       <c r="C77" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D77" t="n">
         <v>18</v>
@@ -2735,10 +2735,10 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>555</v>
+        <v>541</v>
       </c>
       <c r="C78" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D78" t="n">
         <v>18</v>
@@ -2759,57 +2759,57 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>AJO</t>
+          <t>OTROS CITRICOS</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="C79" t="n">
-        <v>49</v>
+        <v>274</v>
       </c>
       <c r="D79" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E79" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="F79" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="G79" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>OTROS CITRICOS</t>
+          <t>AJO</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C80" t="n">
-        <v>273</v>
+        <v>48</v>
       </c>
       <c r="D80" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E80" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="F80" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="G80" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H80" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="C83" t="n">
         <v>89</v>
@@ -2903,7 +2903,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="C84" t="n">
         <v>36</v>
@@ -2959,7 +2959,7 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C86" t="n">
         <v>55</v>
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C88" t="n">
         <v>60</v>
@@ -3151,48 +3151,48 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>BREVO</t>
+          <t>TABACO</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="C93" t="n">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="D93" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E93" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F93" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="G93" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H93" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ULLUCO</t>
+          <t>BREVO</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C94" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="D94" t="n">
         <v>18</v>
       </c>
       <c r="E94" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F94" t="n">
         <v>0</v>
@@ -3207,107 +3207,107 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>TABACO</t>
+          <t>ULLUCO</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="C95" t="n">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="D95" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E95" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="F95" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="G95" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H95" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ESPINACA</t>
+          <t>FLORES Y FOLLAJES</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>330</v>
+        <v>312</v>
       </c>
       <c r="C96" t="n">
-        <v>32</v>
+        <v>76</v>
       </c>
       <c r="D96" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E96" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F96" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>FLORES Y FOLLAJES</t>
+          <t>LIMA</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C97" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D97" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E97" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F97" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>LIMA</t>
+          <t>GUANDUL</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="C98" t="n">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="D98" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E98" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="F98" t="n">
-        <v>11</v>
+        <v>272</v>
       </c>
       <c r="G98" t="n">
         <v>0</v>
@@ -3319,23 +3319,23 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>GUANDUL</t>
+          <t>TANGELO</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C99" t="n">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="D99" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E99" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F99" t="n">
-        <v>273</v>
+        <v>12</v>
       </c>
       <c r="G99" t="n">
         <v>0</v>
@@ -3347,23 +3347,23 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>TANGELO</t>
+          <t>CIMARRON</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="C100" t="n">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="D100" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E100" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F100" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G100" t="n">
         <v>0</v>
@@ -3375,20 +3375,20 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CIMARRON</t>
+          <t>ESPINACA</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C101" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D101" t="n">
         <v>18</v>
       </c>
       <c r="E101" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F101" t="n">
         <v>0</v>
@@ -3431,23 +3431,23 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ARAZA</t>
+          <t>APIO</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C103" t="n">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="D103" t="n">
         <v>18</v>
       </c>
       <c r="E103" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F103" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G103" t="n">
         <v>0</v>
@@ -3459,20 +3459,20 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>BADEA</t>
+          <t>ARAZA</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="C104" t="n">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="D104" t="n">
         <v>18</v>
       </c>
       <c r="E104" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F104" t="n">
         <v>0</v>
@@ -3487,23 +3487,23 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>APIO</t>
+          <t>BADEA</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C105" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D105" t="n">
         <v>18</v>
       </c>
       <c r="E105" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F105" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G105" t="n">
         <v>0</v>
@@ -3543,23 +3543,23 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>AVENA</t>
+          <t>CALABACIN, CALABAZA</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="C107" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D107" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E107" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F107" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G107" t="n">
         <v>0</v>
@@ -3571,23 +3571,23 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CALABACIN, CALABAZA</t>
+          <t>MAIZ FORRAJERO</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="C108" t="n">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="D108" t="n">
+        <v>12</v>
+      </c>
+      <c r="E108" t="n">
+        <v>12</v>
+      </c>
+      <c r="F108" t="n">
         <v>6</v>
-      </c>
-      <c r="E108" t="n">
-        <v>10</v>
-      </c>
-      <c r="F108" t="n">
-        <v>9</v>
       </c>
       <c r="G108" t="n">
         <v>0</v>
@@ -3599,23 +3599,23 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MAIZ FORRAJERO</t>
+          <t>AVENA</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="C109" t="n">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="D109" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E109" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F109" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G109" t="n">
         <v>0</v>
@@ -3687,10 +3687,10 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C112" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D112" t="n">
         <v>11</v>
@@ -3851,57 +3851,57 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ASAI</t>
+          <t>ACHIOTE</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C118" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="D118" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E118" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F118" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="G118" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ACHIOTE</t>
+          <t>PERA</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="C119" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="D119" t="n">
         <v>18</v>
       </c>
       <c r="E119" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F119" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="G119" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H119" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120">
@@ -3911,7 +3911,7 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C120" t="n">
         <v>13</v>
@@ -3935,20 +3935,20 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>PERA</t>
+          <t>ASAI</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C121" t="n">
+        <v>20</v>
+      </c>
+      <c r="D121" t="n">
         <v>16</v>
       </c>
-      <c r="D121" t="n">
-        <v>18</v>
-      </c>
       <c r="E121" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F121" t="n">
         <v>0</v>
@@ -3963,20 +3963,20 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>MANGOSTINO</t>
+          <t>PALMITO</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C122" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D122" t="n">
         <v>18</v>
       </c>
       <c r="E122" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F122" t="n">
         <v>0</v>
@@ -3991,20 +3991,20 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>PALMITO</t>
+          <t>PIMIENTA</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C123" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D123" t="n">
         <v>18</v>
       </c>
       <c r="E123" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F123" t="n">
         <v>0</v>
@@ -4019,20 +4019,20 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>PIMIENTA</t>
+          <t>MANGOSTINO</t>
         </is>
       </c>
       <c r="B124" t="n">
         <v>113</v>
       </c>
       <c r="C124" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D124" t="n">
         <v>18</v>
       </c>
       <c r="E124" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F124" t="n">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>NABO</t>
+          <t>LIMONARIA</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C147" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D147" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E147" t="n">
         <v>3</v>
@@ -4691,23 +4691,23 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>FLOR DE JAMAICA</t>
+          <t>NABO</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C148" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D148" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E148" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F148" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G148" t="n">
         <v>0</v>
@@ -4719,23 +4719,23 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>LIMONARIA</t>
+          <t>FLOR DE JAMAICA</t>
         </is>
       </c>
       <c r="B149" t="n">
         <v>47</v>
       </c>
       <c r="C149" t="n">
+        <v>15</v>
+      </c>
+      <c r="D149" t="n">
+        <v>9</v>
+      </c>
+      <c r="E149" t="n">
         <v>6</v>
       </c>
-      <c r="D149" t="n">
-        <v>16</v>
-      </c>
-      <c r="E149" t="n">
-        <v>3</v>
-      </c>
       <c r="F149" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G149" t="n">
         <v>0</v>
@@ -4919,16 +4919,16 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C156" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D156" t="n">
         <v>17</v>
       </c>
       <c r="E156" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F156" t="n">
         <v>0</v>
@@ -5115,7 +5115,7 @@
         </is>
       </c>
       <c r="B163" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C163" t="n">
         <v>6</v>
@@ -5251,17 +5251,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>FRAMBUESA</t>
+          <t>PLANTAS AROMATICAS Y MEDICINALES</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C168" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D168" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E168" t="n">
         <v>2</v>
@@ -5279,23 +5279,23 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>CANA FLECHA</t>
+          <t>EUCALIPTO BABY BLUE</t>
         </is>
       </c>
       <c r="B169" t="n">
         <v>28</v>
       </c>
       <c r="C169" t="n">
+        <v>5</v>
+      </c>
+      <c r="D169" t="n">
+        <v>12</v>
+      </c>
+      <c r="E169" t="n">
         <v>3</v>
       </c>
-      <c r="D169" t="n">
-        <v>10</v>
-      </c>
-      <c r="E169" t="n">
-        <v>2</v>
-      </c>
       <c r="F169" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="G169" t="n">
         <v>0</v>
@@ -5307,23 +5307,23 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>EUCALIPTO BABY BLUE</t>
+          <t>CANA FLECHA</t>
         </is>
       </c>
       <c r="B170" t="n">
         <v>28</v>
       </c>
       <c r="C170" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D170" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E170" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F170" t="n">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="G170" t="n">
         <v>0</v>
@@ -5363,17 +5363,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>PLANTAS AROMATICAS Y MEDICINALES</t>
+          <t>FRAMBUESA</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C172" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D172" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E172" t="n">
         <v>2</v>
@@ -5475,23 +5475,23 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>RUDA</t>
+          <t>PAPAYUELA -BABACO</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C176" t="n">
+        <v>5</v>
+      </c>
+      <c r="D176" t="n">
         <v>6</v>
       </c>
-      <c r="D176" t="n">
-        <v>15</v>
-      </c>
       <c r="E176" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F176" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G176" t="n">
         <v>0</v>
@@ -5531,23 +5531,23 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>PAPAYUELA -BABACO</t>
+          <t>RUDA</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C178" t="n">
         <v>5</v>
       </c>
       <c r="D178" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E178" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F178" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G178" t="n">
         <v>0</v>
@@ -5671,20 +5671,20 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>CAIMO</t>
+          <t>GIRASOL</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C183" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D183" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E183" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F183" t="n">
         <v>0</v>
@@ -5699,23 +5699,23 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>GIRASOL</t>
+          <t>CEBOLLIN</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C184" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D184" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E184" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F184" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G184" t="n">
         <v>0</v>
@@ -5727,23 +5727,23 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>CEBOLLIN</t>
+          <t>MENTA</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C185" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D185" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E185" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F185" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G185" t="n">
         <v>0</v>
@@ -5755,17 +5755,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>AGUAJE</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C186" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D186" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E186" t="n">
         <v>1</v>
@@ -5811,23 +5811,23 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>AGUAJE</t>
+          <t>COROZO</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C188" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D188" t="n">
+        <v>10</v>
+      </c>
+      <c r="E188" t="n">
+        <v>3</v>
+      </c>
+      <c r="F188" t="n">
         <v>7</v>
-      </c>
-      <c r="E188" t="n">
-        <v>1</v>
-      </c>
-      <c r="F188" t="n">
-        <v>0</v>
       </c>
       <c r="G188" t="n">
         <v>0</v>
@@ -5839,20 +5839,20 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>MENTA</t>
+          <t>MANZANILLA</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C189" t="n">
+        <v>5</v>
+      </c>
+      <c r="D189" t="n">
+        <v>7</v>
+      </c>
+      <c r="E189" t="n">
         <v>3</v>
-      </c>
-      <c r="D189" t="n">
-        <v>13</v>
-      </c>
-      <c r="E189" t="n">
-        <v>1</v>
       </c>
       <c r="F189" t="n">
         <v>0</v>
@@ -5867,23 +5867,23 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>MANZANILLA</t>
+          <t>NONI</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C190" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D190" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E190" t="n">
         <v>3</v>
       </c>
       <c r="F190" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G190" t="n">
         <v>0</v>
@@ -5895,23 +5895,23 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>COROZO</t>
+          <t>CHAMPINON</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C191" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D191" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E191" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F191" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G191" t="n">
         <v>0</v>
@@ -5923,23 +5923,23 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>LAUREL</t>
+          <t>OREGANO</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C192" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D192" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E192" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F192" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G192" t="n">
         <v>0</v>
@@ -5951,23 +5951,23 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>OREGANO</t>
+          <t>POLEO</t>
         </is>
       </c>
       <c r="B193" t="n">
         <v>12</v>
       </c>
       <c r="C193" t="n">
+        <v>2</v>
+      </c>
+      <c r="D193" t="n">
         <v>5</v>
       </c>
-      <c r="D193" t="n">
-        <v>8</v>
-      </c>
       <c r="E193" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F193" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G193" t="n">
         <v>0</v>
@@ -5979,17 +5979,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>POLEO</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="B194" t="n">
         <v>12</v>
       </c>
       <c r="C194" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D194" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E194" t="n">
         <v>1</v>
@@ -6007,20 +6007,20 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>MORINGA</t>
+          <t>CAIMO</t>
         </is>
       </c>
       <c r="B195" t="n">
         <v>12</v>
       </c>
       <c r="C195" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D195" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E195" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F195" t="n">
         <v>0</v>
@@ -6035,11 +6035,11 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>CHAMPINON</t>
+          <t>PUERRO</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C196" t="n">
         <v>3</v>
@@ -6048,7 +6048,7 @@
         <v>6</v>
       </c>
       <c r="E196" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F196" t="n">
         <v>0</v>
@@ -6063,23 +6063,23 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>NONI</t>
+          <t>ASPARRAGUS</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C197" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D197" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E197" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F197" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G197" t="n">
         <v>0</v>
@@ -6091,48 +6091,48 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>PUERRO</t>
+          <t>MILLO</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C198" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D198" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E198" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F198" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G198" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H198" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>ASPARRAGUS</t>
+          <t>PLANTAS MEDICINALES</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C199" t="n">
+        <v>4</v>
+      </c>
+      <c r="D199" t="n">
+        <v>7</v>
+      </c>
+      <c r="E199" t="n">
         <v>3</v>
-      </c>
-      <c r="D199" t="n">
-        <v>6</v>
-      </c>
-      <c r="E199" t="n">
-        <v>2</v>
       </c>
       <c r="F199" t="n">
         <v>0</v>
@@ -6147,48 +6147,48 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>MILLO</t>
+          <t>COCONA</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C200" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D200" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E200" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F200" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G200" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H200" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>PLANTAS MEDICINALES</t>
+          <t>AMARANTO</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C201" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D201" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E201" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F201" t="n">
         <v>0</v>
@@ -6231,17 +6231,17 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>AMARANTO</t>
+          <t>PALMA ROBELINA</t>
         </is>
       </c>
       <c r="B203" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C203" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D203" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E203" t="n">
         <v>1</v>
@@ -6259,20 +6259,20 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>COCONA</t>
+          <t>CENTENO</t>
         </is>
       </c>
       <c r="B204" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C204" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D204" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E204" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F204" t="n">
         <v>0</v>
@@ -6343,17 +6343,17 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>PALMA ROBELINA</t>
+          <t>ACHICORIA</t>
         </is>
       </c>
       <c r="B207" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C207" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D207" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E207" t="n">
         <v>1</v>
@@ -6371,20 +6371,20 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>CENTENO</t>
+          <t>MIMBRE</t>
         </is>
       </c>
       <c r="B208" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C208" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D208" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E208" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F208" t="n">
         <v>0</v>
@@ -6399,7 +6399,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>ACHICORIA</t>
+          <t>OTROS CULTIVOS TROPICALES TRADICIONALES</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -6409,13 +6409,13 @@
         <v>2</v>
       </c>
       <c r="D209" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E209" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F209" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G209" t="n">
         <v>0</v>
@@ -6427,20 +6427,20 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>MIMBRE</t>
+          <t>OTROS CADUCIFOLIOS</t>
         </is>
       </c>
       <c r="B210" t="n">
         <v>6</v>
       </c>
       <c r="C210" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D210" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E210" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F210" t="n">
         <v>0</v>
@@ -6455,7 +6455,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>OTROS CADUCIFOLIOS</t>
+          <t>CHONQUE</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -6465,7 +6465,7 @@
         <v>3</v>
       </c>
       <c r="D211" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E211" t="n">
         <v>2</v>
@@ -6483,23 +6483,23 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>OTROS CULTIVOS TROPICALES TRADICIONALES</t>
+          <t>RUBA</t>
         </is>
       </c>
       <c r="B212" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C212" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D212" t="n">
         <v>4</v>
       </c>
       <c r="E212" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F212" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G212" t="n">
         <v>0</v>
@@ -6511,23 +6511,23 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>CHONQUE</t>
+          <t>PALMA AMARGA</t>
         </is>
       </c>
       <c r="B213" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C213" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D213" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E213" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F213" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G213" t="n">
         <v>0</v>
@@ -6567,11 +6567,11 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>RUBA</t>
+          <t>LAUREL</t>
         </is>
       </c>
       <c r="B215" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C215" t="n">
         <v>1</v>
@@ -6595,23 +6595,23 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>PALMA AMARGA</t>
+          <t>TORONJIL</t>
         </is>
       </c>
       <c r="B216" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C216" t="n">
         <v>1</v>
       </c>
       <c r="D216" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E216" t="n">
         <v>1</v>
       </c>
       <c r="F216" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G216" t="n">
         <v>0</v>
@@ -6651,7 +6651,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>TORONJIL</t>
+          <t>OLIVO</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -6667,7 +6667,7 @@
         <v>1</v>
       </c>
       <c r="F218" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G218" t="n">
         <v>0</v>
@@ -6707,20 +6707,20 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>OLIVO</t>
+          <t>FITOSPORUM</t>
         </is>
       </c>
       <c r="B220" t="n">
         <v>4</v>
       </c>
       <c r="C220" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D220" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E220" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F220" t="n">
         <v>0</v>
@@ -6735,14 +6735,14 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>ALCACHOFA</t>
+          <t>CORDELINE CINTA</t>
         </is>
       </c>
       <c r="B221" t="n">
         <v>4</v>
       </c>
       <c r="C221" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D221" t="n">
         <v>2</v>
@@ -6791,17 +6791,17 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>CORDELINE CINTA</t>
+          <t>ENELDO</t>
         </is>
       </c>
       <c r="B223" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C223" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D223" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E223" t="n">
         <v>1</v>
@@ -6819,20 +6819,20 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>FITOSPORUM</t>
+          <t>LENTEJA</t>
         </is>
       </c>
       <c r="B224" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C224" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D224" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E224" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F224" t="n">
         <v>0</v>
@@ -6847,7 +6847,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>ENELDO</t>
+          <t>ALGARROBO</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -6875,7 +6875,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>ALGARROBO</t>
+          <t>CARAMBOLO</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -6931,17 +6931,17 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>CARAMBOLO</t>
+          <t>PROTEA</t>
         </is>
       </c>
       <c r="B228" t="n">
         <v>3</v>
       </c>
       <c r="C228" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D228" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E228" t="n">
         <v>1</v>
@@ -6959,20 +6959,20 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>POMARROSA</t>
+          <t>COCCULUS</t>
         </is>
       </c>
       <c r="B229" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C229" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D229" t="n">
         <v>2</v>
       </c>
       <c r="E229" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F229" t="n">
         <v>0</v>
@@ -6987,11 +6987,11 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>LENTEJA</t>
+          <t>ANIS</t>
         </is>
       </c>
       <c r="B230" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C230" t="n">
         <v>1</v>
@@ -7015,17 +7015,17 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>PROTEA</t>
+          <t>POMARROSA</t>
         </is>
       </c>
       <c r="B231" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C231" t="n">
         <v>2</v>
       </c>
       <c r="D231" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E231" t="n">
         <v>1</v>
@@ -7043,20 +7043,20 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>ANIS</t>
+          <t>HIBIAS, OCAS</t>
         </is>
       </c>
       <c r="B232" t="n">
         <v>2</v>
       </c>
       <c r="C232" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D232" t="n">
         <v>2</v>
       </c>
       <c r="E232" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F232" t="n">
         <v>0</v>
@@ -7071,7 +7071,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>LIMONIUM</t>
+          <t>HIERBABUENA</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -7099,20 +7099,20 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>HIBIAS, OCAS</t>
+          <t>LIMONIUM</t>
         </is>
       </c>
       <c r="B234" t="n">
         <v>2</v>
       </c>
       <c r="C234" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D234" t="n">
         <v>2</v>
       </c>
       <c r="E234" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F234" t="n">
         <v>0</v>
@@ -7127,20 +7127,20 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>HIERBABUENA</t>
+          <t>UMARI</t>
         </is>
       </c>
       <c r="B235" t="n">
         <v>2</v>
       </c>
       <c r="C235" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D235" t="n">
         <v>2</v>
       </c>
       <c r="E235" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F235" t="n">
         <v>0</v>
@@ -7183,20 +7183,20 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>UMARI</t>
+          <t>BORE</t>
         </is>
       </c>
       <c r="B237" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C237" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D237" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E237" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F237" t="n">
         <v>0</v>
@@ -7211,17 +7211,17 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>COCCULUS</t>
+          <t>CALENDULA</t>
         </is>
       </c>
       <c r="B238" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C238" t="n">
         <v>1</v>
       </c>
       <c r="D238" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E238" t="n">
         <v>1</v>
@@ -7351,7 +7351,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>BORE</t>
+          <t>ALCACHOFA</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -7407,7 +7407,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>CALENDULA</t>
+          <t>MORINGA</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -7471,7 +7471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7482,7 +7482,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>filas</t>
+          <t>filas_eliminadas</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>filas_restantes</t>
         </is>
       </c>
     </row>
@@ -7493,57 +7498,75 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
         <v>351920</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Se descarta 2006 (no pertenece al rango)</t>
+          <t>Se descarta 2006 (fuera del rango 2007-2024)</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>4072</v>
       </c>
+      <c r="C3" t="n">
+        <v>347848</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sin área cosechada (&lt;=0 o vacía)</t>
+          <t>Sin area cosechada (&lt;=0 o vacia)</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>9020</v>
       </c>
+      <c r="C4" t="n">
+        <v>338828</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Área cosechada &gt; sembrada + 10%</t>
+          <t>Sin produccion (&lt;=0 o vacia)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8683</v>
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>338828</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Rendimientos atípicos (3 x IQR en log, por cultivo)</t>
+          <t>Cosechada &gt; sembrada (+10% tolerancia)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1130</v>
+        <v>8683</v>
+      </c>
+      <c r="C6" t="n">
+        <v>330145</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Filas limpias finales</t>
+          <t>Rendimientos atipicos (3 x IQR en log; limites con 2007-2018)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>329015</v>
+        <v>1379</v>
+      </c>
+      <c r="C7" t="n">
+        <v>328766</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corregir ciclo y region Caribe en el pipeline EVA; agregar pruebas, README y requirements en UTF-8
</commit_message>
<xml_diff>
--- a/ml/reports/conteo_cultivos_EVA.xlsx
+++ b/ml/reports/conteo_cultivos_EVA.xlsx
@@ -479,7 +479,7 @@
         <v>33</v>
       </c>
       <c r="F2" t="n">
-        <v>8341</v>
+        <v>8367</v>
       </c>
       <c r="G2" t="n">
         <v>1839</v>
@@ -507,7 +507,7 @@
         <v>33</v>
       </c>
       <c r="F3" t="n">
-        <v>4008</v>
+        <v>4028</v>
       </c>
       <c r="G3" t="n">
         <v>928</v>
@@ -535,7 +535,7 @@
         <v>19</v>
       </c>
       <c r="F4" t="n">
-        <v>1733</v>
+        <v>1751</v>
       </c>
       <c r="G4" t="n">
         <v>289</v>
@@ -619,7 +619,7 @@
         <v>33</v>
       </c>
       <c r="F2" t="n">
-        <v>8341</v>
+        <v>8367</v>
       </c>
       <c r="G2" t="n">
         <v>1839</v>
@@ -675,7 +675,7 @@
         <v>33</v>
       </c>
       <c r="F4" t="n">
-        <v>4008</v>
+        <v>4028</v>
       </c>
       <c r="G4" t="n">
         <v>928</v>
@@ -731,7 +731,7 @@
         <v>33</v>
       </c>
       <c r="F6" t="n">
-        <v>2313</v>
+        <v>2333</v>
       </c>
       <c r="G6" t="n">
         <v>618</v>
@@ -899,7 +899,7 @@
         <v>30</v>
       </c>
       <c r="F12" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="G12" t="n">
         <v>145</v>
@@ -983,7 +983,7 @@
         <v>32</v>
       </c>
       <c r="F15" t="n">
-        <v>953</v>
+        <v>960</v>
       </c>
       <c r="G15" t="n">
         <v>121</v>
@@ -1011,7 +1011,7 @@
         <v>30</v>
       </c>
       <c r="F16" t="n">
-        <v>1616</v>
+        <v>1624</v>
       </c>
       <c r="G16" t="n">
         <v>268</v>
@@ -1095,7 +1095,7 @@
         <v>32</v>
       </c>
       <c r="F19" t="n">
-        <v>919</v>
+        <v>926</v>
       </c>
       <c r="G19" t="n">
         <v>161</v>
@@ -1151,7 +1151,7 @@
         <v>31</v>
       </c>
       <c r="F21" t="n">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="G21" t="n">
         <v>70</v>
@@ -1179,7 +1179,7 @@
         <v>29</v>
       </c>
       <c r="F22" t="n">
-        <v>2296</v>
+        <v>2308</v>
       </c>
       <c r="G22" t="n">
         <v>207</v>
@@ -1207,7 +1207,7 @@
         <v>27</v>
       </c>
       <c r="F23" t="n">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -1235,7 +1235,7 @@
         <v>25</v>
       </c>
       <c r="F24" t="n">
-        <v>1591</v>
+        <v>1600</v>
       </c>
       <c r="G24" t="n">
         <v>407</v>
@@ -1291,7 +1291,7 @@
         <v>33</v>
       </c>
       <c r="F26" t="n">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="G26" t="n">
         <v>49</v>
@@ -1347,7 +1347,7 @@
         <v>22</v>
       </c>
       <c r="F28" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G28" t="n">
         <v>12</v>
@@ -1375,7 +1375,7 @@
         <v>27</v>
       </c>
       <c r="F29" t="n">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -1487,7 +1487,7 @@
         <v>29</v>
       </c>
       <c r="F33" t="n">
-        <v>488</v>
+        <v>507</v>
       </c>
       <c r="G33" t="n">
         <v>19</v>
@@ -1543,7 +1543,7 @@
         <v>24</v>
       </c>
       <c r="F35" t="n">
-        <v>1496</v>
+        <v>1506</v>
       </c>
       <c r="G35" t="n">
         <v>182</v>
@@ -1627,7 +1627,7 @@
         <v>27</v>
       </c>
       <c r="F38" t="n">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="G38" t="n">
         <v>196</v>
@@ -1655,7 +1655,7 @@
         <v>27</v>
       </c>
       <c r="F39" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="G39" t="n">
         <v>4</v>
@@ -1683,7 +1683,7 @@
         <v>28</v>
       </c>
       <c r="F40" t="n">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="G40" t="n">
         <v>26</v>
@@ -1711,7 +1711,7 @@
         <v>19</v>
       </c>
       <c r="F41" t="n">
-        <v>1733</v>
+        <v>1751</v>
       </c>
       <c r="G41" t="n">
         <v>289</v>
@@ -1739,7 +1739,7 @@
         <v>28</v>
       </c>
       <c r="F42" t="n">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="G42" t="n">
         <v>52</v>
@@ -1991,7 +1991,7 @@
         <v>18</v>
       </c>
       <c r="F51" t="n">
-        <v>607</v>
+        <v>619</v>
       </c>
       <c r="G51" t="n">
         <v>117</v>
@@ -2355,7 +2355,7 @@
         <v>12</v>
       </c>
       <c r="F64" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G64" t="n">
         <v>0</v>
@@ -2495,7 +2495,7 @@
         <v>14</v>
       </c>
       <c r="F69" t="n">
-        <v>491</v>
+        <v>498</v>
       </c>
       <c r="G69" t="n">
         <v>65</v>
@@ -2523,7 +2523,7 @@
         <v>13</v>
       </c>
       <c r="F70" t="n">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
@@ -3531,7 +3531,7 @@
         <v>14</v>
       </c>
       <c r="F106" t="n">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="G106" t="n">
         <v>6</v>
@@ -4287,7 +4287,7 @@
         <v>13</v>
       </c>
       <c r="F133" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G133" t="n">
         <v>0</v>
@@ -5015,7 +5015,7 @@
         <v>4</v>
       </c>
       <c r="F159" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G159" t="n">
         <v>0</v>

</xml_diff>